<commit_message>
New traynelis replica 9-26
</commit_message>
<xml_diff>
--- a/Scripts/Experiments/Creating_NSFA_Debugger/testing_NSFA_matrix.xlsx
+++ b/Scripts/Experiments/Creating_NSFA_Debugger/testing_NSFA_matrix.xlsx
@@ -40,7 +40,7 @@
     <t>template_max</t>
   </si>
   <si>
-    <t>EPSCs</t>
+    <t>Sheet1</t>
   </si>
   <si>
     <t>peak</t>
@@ -453,16 +453,16 @@
         <v>11</v>
       </c>
       <c r="F2">
-        <v>0.5345550586340194</v>
+        <v>1.463570164458643</v>
       </c>
       <c r="G2">
-        <v>0.8738911952513212</v>
+        <v>1.463570164458643</v>
       </c>
       <c r="H2">
-        <v>434.9819708843859</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>208.8630303030311</v>
+        <v>84.57485148514851</v>
       </c>
     </row>
   </sheetData>

</xml_diff>